<commit_message>
Add archive_index.xlsx with conditional dropdowns
https://claude.ai/code/session_01LG1wPERtMFPnjz7WXpbQZ4
</commit_message>
<xml_diff>
--- a/archive_index.xlsx
+++ b/archive_index.xlsx
@@ -11,15 +11,24 @@
     <sheet name="Lists" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="seasons">Lists!$A$2:$A$7</definedName>
-    <definedName name="categories">Lists!$B$2:$B$6</definedName>
-    <definedName name="adv">Lists!$C$2:$C$5</definedName>
-    <definedName name="col">Lists!$D$2:$D$6</definedName>
-    <definedName name="edi">Lists!$E$2:$E$10</definedName>
-    <definedName name="inv">Lists!$F$2:$F$3</definedName>
-    <definedName name="eph">Lists!$G$2:$G$5</definedName>
-    <definedName name="desc_adv">Lists!$H$2:$H$9</definedName>
-    <definedName name="desc_col">Lists!$I$2:$I$4</definedName>
+    <definedName name="years">Lists!$A$2:$A$60</definedName>
+    <definedName name="seasons">Lists!$B$2:$B$7</definedName>
+    <definedName name="categories">Lists!$C$2:$C$6</definedName>
+    <definedName name="adv">Lists!$D$2:$D$5</definedName>
+    <definedName name="col">Lists!$E$2:$E$6</definedName>
+    <definedName name="edi">Lists!$F$2:$F$10</definedName>
+    <definedName name="inv">Lists!$G$2:$G$3</definedName>
+    <definedName name="eph">Lists!$H$2:$H$5</definedName>
+    <definedName name="desc_adv">Lists!$I$2:$I$9</definedName>
+    <definedName name="desc_col">Lists!$J$2:$J$4</definedName>
+    <definedName name="fragrance">Lists!$K$2:$K$13</definedName>
+    <definedName name="jeans">Lists!$L$2:$L$5</definedName>
+    <definedName name="underwear">Lists!$M$2:$M$4</definedName>
+    <definedName name="eyewear">Lists!$N$2:$N$2</definedName>
+    <definedName name="denim">Lists!$O$2:$O$2</definedName>
+    <definedName name="accessories">Lists!$P$2:$P$2</definedName>
+    <definedName name="shoes">Lists!$Q$2:$Q$2</definedName>
+    <definedName name="rtw">Lists!$R$2:$R$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -434,7 +443,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
@@ -588,7 +597,10 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="6">
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=years</formula1>
+    </dataValidation>
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=seasons</formula1>
     </dataValidation>
@@ -601,6 +613,9 @@
     <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=INDIRECT("desc_"&amp;$D2)</formula1>
     </dataValidation>
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=INDIRECT(SUBSTITUTE($G2," ","_"))</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -612,301 +627,861 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:R60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>seasons</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>categories</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>adv</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>col</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>edi</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>inv</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>eph</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>desc_adv</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>desc_col</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>fragrance</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>jeans</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>underwear</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>eyewear</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>denim</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>accessories</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>shoes</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>rtw</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>1968</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>ss</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>adv</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>print</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>rtw-w</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>vogue-us</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>show</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>backstage</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>fragrance</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>runway</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>obsession</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>are you wearing any</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>ck underwear</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>ck eyewear</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>ck denim</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>ck accessories</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>ck shoes</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>ck rtw</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>1969</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>fw</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>col</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>ooh</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>rtw-m</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>vogue-it</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>event</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>fitting</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>jeans</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>lookbook</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>eternity</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>nothing comes between me</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>my calvins</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>1970</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>aw</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>edi</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>digital</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>couture</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>vogue-paris</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>bts</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>underwear</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>catalog</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ck one</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>just the way you are</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>i __ my calvins</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>1971</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>cruise</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>inv</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>video</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>denim</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>harpers</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>portrait</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>eyewear</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>escape</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>ck jeans</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>1972</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>pre-fall</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>eph</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>underwear</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>iD</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>denim</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>contradiction</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>1973</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>resort</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>dazed</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>accessories</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>truth</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="E8" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1974</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>interview</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>shoes</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>be</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="E9" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>wmag</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>rtw</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>euphoria</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="E10" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1976</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>numero</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ck2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1977</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>eternity moment</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1978</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1979</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ck all</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1980</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1981</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1982</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1983</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1984</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1985</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1986</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1987</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1988</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1989</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1991</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1996</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1999</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2002</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove venue and add dropdowns for all creative roles
https://claude.ai/code/session_01LG1wPERtMFPnjz7WXpbQZ4
</commit_message>
<xml_diff>
--- a/archive_index.xlsx
+++ b/archive_index.xlsx
@@ -29,6 +29,19 @@
     <definedName name="accessories">Lists!$P$2:$P$2</definedName>
     <definedName name="shoes">Lists!$Q$2:$Q$2</definedName>
     <definedName name="rtw">Lists!$R$2:$R$2</definedName>
+    <definedName name="photographers">Lists!$S$2:$S$31</definedName>
+    <definedName name="directors">Lists!$T$2:$T$16</definedName>
+    <definedName name="models">Lists!$U$2:$U$27</definedName>
+    <definedName name="stylists">Lists!$V$2:$V$13</definedName>
+    <definedName name="hair_list">Lists!$W$2:$W$10</definedName>
+    <definedName name="makeup_list">Lists!$X$2:$X$11</definedName>
+    <definedName name="art_directors">Lists!$Y$2:$Y$6</definedName>
+    <definedName name="creative_directors">Lists!$Z$2:$Z$8</definedName>
+    <definedName name="set_designers">Lists!$AA$2:$AA$6</definedName>
+    <definedName name="casting_directors">Lists!$AB$2:$AB$6</definedName>
+    <definedName name="production_companies">Lists!$AC$2:$AC$7</definedName>
+    <definedName name="agencies">Lists!$AD$2:$AD$7</definedName>
+    <definedName name="publications">Lists!$AE$2:$AE$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -441,27 +454,26 @@
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="30" customWidth="1" min="25" max="25"/>
-    <col width="24" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="30" customWidth="1" min="24" max="24"/>
+    <col width="24" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,129 +504,163 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>venue</t>
+          <t>description</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>campaign</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>campaign</t>
+          <t>photographer</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>photographer</t>
+          <t>director</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>director</t>
+          <t>producer</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>producer</t>
+          <t>production_company</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>production_company</t>
+          <t>model</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>stylist</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>stylist</t>
+          <t>art_director</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>art_director</t>
+          <t>creative_director</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>creative_director</t>
+          <t>hair</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>hair</t>
+          <t>makeup</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>makeup</t>
+          <t>set_designer</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>set_designer</t>
+          <t>casting_director</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>casting_director</t>
+          <t>agency</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>agency</t>
+          <t>publication</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>publication</t>
+          <t>issue_date</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>issue_date</t>
+          <t>music</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>music</t>
+          <t>source_url</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>source_url</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
           <t>notes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="19">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=years</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=seasons</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=categories</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=photographers</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=directors</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=models</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=stylists</formula1>
+    </dataValidation>
+    <dataValidation sqref="P2:P1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=hair_list</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q2:Q1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=makeup_list</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=art_directors</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=creative_directors</formula1>
+    </dataValidation>
+    <dataValidation sqref="R2:R1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=set_designers</formula1>
+    </dataValidation>
+    <dataValidation sqref="S2:S1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=casting_directors</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=production_companies</formula1>
+    </dataValidation>
+    <dataValidation sqref="T2:T1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=agencies</formula1>
+    </dataValidation>
+    <dataValidation sqref="U2:U1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=publications</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=INDIRECT($D2)</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=INDIRECT("desc_"&amp;$D2)</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=INDIRECT(SUBSTITUTE($G2," ","_"))</formula1>
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=INDIRECT(SUBSTITUTE($F2," ","_"))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -627,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R60"/>
+  <dimension ref="A1:AE60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -721,6 +767,71 @@
           <t>rtw</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>photographers</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>directors</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>models</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>stylists</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>hair_list</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>makeup_list</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>art_directors</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>creative_directors</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>set_designers</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>casting_directors</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>production_companies</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>agencies</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>publications</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -813,6 +924,71 @@
           <t>ck rtw</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Bruce Weber</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Fabien Baron</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Kate Moss</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Camilla Nickerson</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Garren</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Pat McGrath</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Fabien Baron</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Calvin Klein</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Stefan Beckman</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>James Scully</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Baron &amp; Baron</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Baron &amp; Baron</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Vogue US</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -880,6 +1056,71 @@
           <t>my calvins</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Steven Meisel</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>David Fincher</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Christy Turlington</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Joe McKenna</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Guido Palau</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Diane Kendal</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Sam Shahid</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Raf Simons</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Mary Howard</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Piergiorgio Del Moro</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>CDM</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>CDM</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Vogue Italia</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -942,6 +1183,71 @@
           <t>i __ my calvins</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Richard Avedon</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Bruce Weber</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Naomi Campbell</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Karl Templer</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Sam McKnight</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Aaron de Mey</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Tibor Kalman</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Francisco Costa</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Andy Hillman</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>Ashley Brokaw</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Calvin Klein Inc.</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Wieden+Kennedy</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Vogue Paris</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -994,6 +1300,71 @@
           <t>ck jeans</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Herb Ritts</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Sofia Coppola</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Cindy Crawford</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Marie-Amélie Sauvé</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Eugene Souleiman</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Tom Pecheux</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Neville Brody</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Italo Zucchelli</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Piers Hanmer</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>Jess Hallett</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>Hungry Man</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>Mother</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>Harper's Bazaar</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1031,6 +1402,71 @@
           <t>contradiction</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Patrick Demarchelier</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Mario Sorrenti</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Linda Evangelista</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Olivier Rizzo</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Christiaan Houtenbos</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>François Nars</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Peter Saville</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Kevin Carrigan</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Jack Flanagan</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>Anita Bitton</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>RSA Films</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>Laird+Partners</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>i-D</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1058,6 +1494,56 @@
           <t>truth</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Mario Sorrenti</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Steven Meisel</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Brooke Shields</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Alastair McKimm</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Didier Malige</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Kevyn Aucoin</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Pieter Mulier</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>Anonymous Content</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>CKX</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>Dazed</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1080,6 +1566,46 @@
           <t>be</t>
         </is>
       </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>David Sims</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Herb Ritts</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Mark Wahlberg</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Lucinda Chambers</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Julien d'Ys</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Linda Cantello</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Veronica Leoni</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1102,6 +1628,41 @@
           <t>euphoria</t>
         </is>
       </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Mert &amp; Marcus</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Spike Jonze</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Travis Fimmel</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Carlyne Cerf de Dudzeele</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Anthony Turner</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Charlotte Tilbury</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>W Magazine</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1119,6 +1680,41 @@
           <t>ck2</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Steven Klein</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Tony Kaye</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Lara Stone</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Grace Coddington</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Duffy</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Lucia Pieroni</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>Numéro</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1131,6 +1727,36 @@
           <t>eternity moment</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Inez &amp; Vinoodh</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Jonas Åkerlund</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Natalia Vodianova</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Carine Roitfeld</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>Peter Philips</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>Self Service</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1143,6 +1769,31 @@
           <t>free</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Mario Testino</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Mark Romanek</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Jamie Dornan</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Melanie Ward</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1155,6 +1806,31 @@
           <t>ck all</t>
         </is>
       </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Glen Luchford</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Floria Sigismondi</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Gisele Bündchen</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Tonne Goodman</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>Another</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1162,6 +1838,26 @@
           <t>1980</t>
         </is>
       </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Craig McDean</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Steven Klein</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Jessica Stam</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>The Face</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1169,6 +1865,26 @@
           <t>1981</t>
         </is>
       </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Willy Vanderperre</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Mert &amp; Marcus</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Daria Werbowy</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>AnOther Man</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1176,6 +1892,26 @@
           <t>1982</t>
         </is>
       </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Fabien Baron</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Sam Taylor-Johnson</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Edie Campbell</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>GQ</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1183,6 +1919,21 @@
           <t>1983</t>
         </is>
       </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Peter Lindbergh</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Anna Ewers</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>Vanity Fair</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1190,6 +1941,16 @@
           <t>1984</t>
         </is>
       </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Helmut Newton</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Saskia de Brauw</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1197,6 +1958,16 @@
           <t>1985</t>
         </is>
       </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Annie Leibovitz</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Justin Bieber</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1204,6 +1975,16 @@
           <t>1986</t>
         </is>
       </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Nick Knight</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Kendall Jenner</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1211,6 +1992,16 @@
           <t>1987</t>
         </is>
       </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Juergen Teller</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Bella Hadid</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1218,6 +2009,16 @@
           <t>1988</t>
         </is>
       </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Tyrone Lebon</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Lily-Rose Depp</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1225,6 +2026,16 @@
           <t>1989</t>
         </is>
       </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Lachlan Bailey</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>FKA twigs</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1232,6 +2043,16 @@
           <t>1990</t>
         </is>
       </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Cass Bird</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Solange</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1239,6 +2060,16 @@
           <t>1991</t>
         </is>
       </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Harley Weir</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>A$AP Rocky</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1246,6 +2077,16 @@
           <t>1992</t>
         </is>
       </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Daniel Jackson</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Kaia Gerber</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1253,6 +2094,16 @@
           <t>1993</t>
         </is>
       </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Niall McInerney</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Jeremy Allen White</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1260,6 +2111,11 @@
           <t>1994</t>
         </is>
       </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Sølve Sundsbø</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1267,6 +2123,11 @@
           <t>1995</t>
         </is>
       </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Paolo Roversi</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1274,11 +2135,21 @@
           <t>1996</t>
         </is>
       </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Collier Schorr</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
           <t>1997</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Ethan James Green</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make dropdown lists dynamic with OFFSET+COUNTA, add theface to edi
https://claude.ai/code/session_01LG1wPERtMFPnjz7WXpbQZ4
</commit_message>
<xml_diff>
--- a/archive_index.xlsx
+++ b/archive_index.xlsx
@@ -11,37 +11,37 @@
     <sheet name="Lists" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="years">Lists!$A$2:$A$60</definedName>
-    <definedName name="seasons">Lists!$B$2:$B$7</definedName>
-    <definedName name="categories">Lists!$C$2:$C$6</definedName>
-    <definedName name="adv">Lists!$D$2:$D$5</definedName>
-    <definedName name="col">Lists!$E$2:$E$6</definedName>
-    <definedName name="edi">Lists!$F$2:$F$10</definedName>
-    <definedName name="inv">Lists!$G$2:$G$3</definedName>
-    <definedName name="eph">Lists!$H$2:$H$5</definedName>
-    <definedName name="desc_adv">Lists!$I$2:$I$9</definedName>
-    <definedName name="desc_col">Lists!$J$2:$J$4</definedName>
-    <definedName name="fragrance">Lists!$K$2:$K$13</definedName>
-    <definedName name="jeans">Lists!$L$2:$L$5</definedName>
-    <definedName name="underwear">Lists!$M$2:$M$4</definedName>
-    <definedName name="eyewear">Lists!$N$2:$N$2</definedName>
-    <definedName name="denim">Lists!$O$2:$O$2</definedName>
-    <definedName name="accessories">Lists!$P$2:$P$2</definedName>
-    <definedName name="shoes">Lists!$Q$2:$Q$2</definedName>
-    <definedName name="rtw">Lists!$R$2:$R$2</definedName>
-    <definedName name="photographers">Lists!$S$2:$S$31</definedName>
-    <definedName name="directors">Lists!$T$2:$T$16</definedName>
-    <definedName name="models">Lists!$U$2:$U$27</definedName>
-    <definedName name="stylists">Lists!$V$2:$V$13</definedName>
-    <definedName name="hair_list">Lists!$W$2:$W$10</definedName>
-    <definedName name="makeup_list">Lists!$X$2:$X$11</definedName>
-    <definedName name="art_directors">Lists!$Y$2:$Y$6</definedName>
-    <definedName name="creative_directors">Lists!$Z$2:$Z$8</definedName>
-    <definedName name="set_designers">Lists!$AA$2:$AA$6</definedName>
-    <definedName name="casting_directors">Lists!$AB$2:$AB$6</definedName>
-    <definedName name="production_companies">Lists!$AC$2:$AC$7</definedName>
-    <definedName name="agencies">Lists!$AD$2:$AD$7</definedName>
-    <definedName name="publications">Lists!$AE$2:$AE$17</definedName>
+    <definedName name="years">OFFSET(Lists!$A$2,0,0,COUNTA(Lists!$A:$A)-1,1)</definedName>
+    <definedName name="seasons">OFFSET(Lists!$B$2,0,0,COUNTA(Lists!$B:$B)-1,1)</definedName>
+    <definedName name="categories">OFFSET(Lists!$C$2,0,0,COUNTA(Lists!$C:$C)-1,1)</definedName>
+    <definedName name="adv">OFFSET(Lists!$D$2,0,0,COUNTA(Lists!$D:$D)-1,1)</definedName>
+    <definedName name="col">OFFSET(Lists!$E$2,0,0,COUNTA(Lists!$E:$E)-1,1)</definedName>
+    <definedName name="edi">OFFSET(Lists!$F$2,0,0,COUNTA(Lists!$F:$F)-1,1)</definedName>
+    <definedName name="inv">OFFSET(Lists!$G$2,0,0,COUNTA(Lists!$G:$G)-1,1)</definedName>
+    <definedName name="eph">OFFSET(Lists!$H$2,0,0,COUNTA(Lists!$H:$H)-1,1)</definedName>
+    <definedName name="desc_adv">OFFSET(Lists!$I$2,0,0,COUNTA(Lists!$I:$I)-1,1)</definedName>
+    <definedName name="desc_col">OFFSET(Lists!$J$2,0,0,COUNTA(Lists!$J:$J)-1,1)</definedName>
+    <definedName name="fragrance">OFFSET(Lists!$K$2,0,0,COUNTA(Lists!$K:$K)-1,1)</definedName>
+    <definedName name="jeans">OFFSET(Lists!$L$2,0,0,COUNTA(Lists!$L:$L)-1,1)</definedName>
+    <definedName name="underwear">OFFSET(Lists!$M$2,0,0,COUNTA(Lists!$M:$M)-1,1)</definedName>
+    <definedName name="eyewear">OFFSET(Lists!$N$2,0,0,COUNTA(Lists!$N:$N)-1,1)</definedName>
+    <definedName name="denim">OFFSET(Lists!$O$2,0,0,COUNTA(Lists!$O:$O)-1,1)</definedName>
+    <definedName name="accessories">OFFSET(Lists!$P$2,0,0,COUNTA(Lists!$P:$P)-1,1)</definedName>
+    <definedName name="shoes">OFFSET(Lists!$Q$2,0,0,COUNTA(Lists!$Q:$Q)-1,1)</definedName>
+    <definedName name="rtw">OFFSET(Lists!$R$2,0,0,COUNTA(Lists!$R:$R)-1,1)</definedName>
+    <definedName name="photographers">OFFSET(Lists!$S$2,0,0,COUNTA(Lists!$S:$S)-1,1)</definedName>
+    <definedName name="directors">OFFSET(Lists!$T$2,0,0,COUNTA(Lists!$T:$T)-1,1)</definedName>
+    <definedName name="models">OFFSET(Lists!$U$2,0,0,COUNTA(Lists!$U:$U)-1,1)</definedName>
+    <definedName name="stylists">OFFSET(Lists!$V$2,0,0,COUNTA(Lists!$V:$V)-1,1)</definedName>
+    <definedName name="hair_list">OFFSET(Lists!$W$2,0,0,COUNTA(Lists!$W:$W)-1,1)</definedName>
+    <definedName name="makeup_list">OFFSET(Lists!$X$2,0,0,COUNTA(Lists!$X:$X)-1,1)</definedName>
+    <definedName name="art_directors">OFFSET(Lists!$Y$2,0,0,COUNTA(Lists!$Y:$Y)-1,1)</definedName>
+    <definedName name="creative_directors">OFFSET(Lists!$Z$2,0,0,COUNTA(Lists!$Z:$Z)-1,1)</definedName>
+    <definedName name="set_designers">OFFSET(Lists!$AA$2,0,0,COUNTA(Lists!$AA:$AA)-1,1)</definedName>
+    <definedName name="casting_directors">OFFSET(Lists!$AB$2,0,0,COUNTA(Lists!$AB:$AB)-1,1)</definedName>
+    <definedName name="production_companies">OFFSET(Lists!$AC$2,0,0,COUNTA(Lists!$AC:$AC)-1,1)</definedName>
+    <definedName name="agencies">OFFSET(Lists!$AD$2,0,0,COUNTA(Lists!$AD:$AD)-1,1)</definedName>
+    <definedName name="publications">OFFSET(Lists!$AE$2,0,0,COUNTA(Lists!$AE:$AE)-1,1)</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1722,6 +1722,11 @@
           <t>1977</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>theface</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>eternity moment</t>

</xml_diff>

<commit_message>
Store years as integers to avoid Excel text-format warning
https://claude.ai/code/session_01LG1wPERtMFPnjz7WXpbQZ4
</commit_message>
<xml_diff>
--- a/archive_index.xlsx
+++ b/archive_index.xlsx
@@ -834,10 +834,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1968</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1968</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -991,10 +989,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1969</t>
-        </is>
+      <c r="A3" t="n">
+        <v>1969</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1123,10 +1119,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1970</t>
-        </is>
+      <c r="A4" t="n">
+        <v>1970</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1250,10 +1244,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1971</t>
-        </is>
+      <c r="A5" t="n">
+        <v>1971</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1367,10 +1359,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1972</t>
-        </is>
+      <c r="A6" t="n">
+        <v>1972</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1469,10 +1459,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1973</t>
-        </is>
+      <c r="A7" t="n">
+        <v>1973</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1546,10 +1534,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1974</t>
-        </is>
+      <c r="A8" t="n">
+        <v>1974</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1608,10 +1594,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1975</t>
-        </is>
+      <c r="A9" t="n">
+        <v>1975</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1665,10 +1649,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>1976</t>
-        </is>
+      <c r="A10" t="n">
+        <v>1976</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1717,10 +1699,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>1977</t>
-        </is>
+      <c r="A11" t="n">
+        <v>1977</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1764,10 +1744,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>1978</t>
-        </is>
+      <c r="A12" t="n">
+        <v>1978</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1801,10 +1779,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>1979</t>
-        </is>
+      <c r="A13" t="n">
+        <v>1979</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1838,10 +1814,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>1980</t>
-        </is>
+      <c r="A14" t="n">
+        <v>1980</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1865,10 +1839,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>1981</t>
-        </is>
+      <c r="A15" t="n">
+        <v>1981</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -1892,10 +1864,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>1982</t>
-        </is>
+      <c r="A16" t="n">
+        <v>1982</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -1919,10 +1889,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>1983</t>
-        </is>
+      <c r="A17" t="n">
+        <v>1983</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
@@ -1941,10 +1909,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>1984</t>
-        </is>
+      <c r="A18" t="n">
+        <v>1984</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -1958,10 +1924,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>1985</t>
-        </is>
+      <c r="A19" t="n">
+        <v>1985</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
@@ -1975,10 +1939,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>1986</t>
-        </is>
+      <c r="A20" t="n">
+        <v>1986</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
@@ -1992,10 +1954,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>1987</t>
-        </is>
+      <c r="A21" t="n">
+        <v>1987</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
@@ -2009,10 +1969,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>1988</t>
-        </is>
+      <c r="A22" t="n">
+        <v>1988</v>
       </c>
       <c r="S22" t="inlineStr">
         <is>
@@ -2026,10 +1984,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>1989</t>
-        </is>
+      <c r="A23" t="n">
+        <v>1989</v>
       </c>
       <c r="S23" t="inlineStr">
         <is>
@@ -2043,10 +1999,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>1990</t>
-        </is>
+      <c r="A24" t="n">
+        <v>1990</v>
       </c>
       <c r="S24" t="inlineStr">
         <is>
@@ -2060,10 +2014,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>1991</t>
-        </is>
+      <c r="A25" t="n">
+        <v>1991</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
@@ -2077,10 +2029,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>1992</t>
-        </is>
+      <c r="A26" t="n">
+        <v>1992</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
@@ -2094,10 +2044,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>1993</t>
-        </is>
+      <c r="A27" t="n">
+        <v>1993</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
@@ -2111,10 +2059,8 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>1994</t>
-        </is>
+      <c r="A28" t="n">
+        <v>1994</v>
       </c>
       <c r="S28" t="inlineStr">
         <is>
@@ -2123,10 +2069,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>1995</t>
-        </is>
+      <c r="A29" t="n">
+        <v>1995</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
@@ -2135,10 +2079,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>1996</t>
-        </is>
+      <c r="A30" t="n">
+        <v>1996</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
@@ -2147,10 +2089,8 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>1997</t>
-        </is>
+      <c r="A31" t="n">
+        <v>1997</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
@@ -2159,206 +2099,148 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>1998</t>
-        </is>
+      <c r="A32" t="n">
+        <v>1998</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>1999</t>
-        </is>
+      <c r="A33" t="n">
+        <v>1999</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
+      <c r="A34" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
+      <c r="A35" t="n">
+        <v>2001</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2002</t>
-        </is>
+      <c r="A36" t="n">
+        <v>2002</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>2003</t>
-        </is>
+      <c r="A37" t="n">
+        <v>2003</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2004</t>
-        </is>
+      <c r="A38" t="n">
+        <v>2004</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2005</t>
-        </is>
+      <c r="A39" t="n">
+        <v>2005</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>2006</t>
-        </is>
+      <c r="A40" t="n">
+        <v>2006</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>2007</t>
-        </is>
+      <c r="A41" t="n">
+        <v>2007</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>2008</t>
-        </is>
+      <c r="A42" t="n">
+        <v>2008</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>2009</t>
-        </is>
+      <c r="A43" t="n">
+        <v>2009</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>2010</t>
-        </is>
+      <c r="A44" t="n">
+        <v>2010</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
+      <c r="A45" t="n">
+        <v>2011</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
+      <c r="A46" t="n">
+        <v>2012</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>2013</t>
-        </is>
+      <c r="A47" t="n">
+        <v>2013</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
+      <c r="A48" t="n">
+        <v>2014</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
+      <c r="A49" t="n">
+        <v>2015</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>2016</t>
-        </is>
+      <c r="A50" t="n">
+        <v>2016</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
+      <c r="A51" t="n">
+        <v>2017</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
+      <c r="A52" t="n">
+        <v>2018</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
+      <c r="A53" t="n">
+        <v>2019</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
+      <c r="A54" t="n">
+        <v>2020</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
+      <c r="A55" t="n">
+        <v>2021</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
+      <c r="A56" t="n">
+        <v>2022</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
+      <c r="A57" t="n">
+        <v>2023</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
+      <c r="A58" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+      <c r="A59" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
+      <c r="A60" t="n">
+        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use Excel Tables for auto-expanding dropdown lists
https://claude.ai/code/session_01LG1wPERtMFPnjz7WXpbQZ4
</commit_message>
<xml_diff>
--- a/archive_index.xlsx
+++ b/archive_index.xlsx
@@ -11,37 +11,37 @@
     <sheet name="Lists" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="years">OFFSET(Lists!$A$2,0,0,COUNTA(Lists!$A:$A)-1,1)</definedName>
-    <definedName name="seasons">OFFSET(Lists!$B$2,0,0,COUNTA(Lists!$B:$B)-1,1)</definedName>
-    <definedName name="categories">OFFSET(Lists!$C$2,0,0,COUNTA(Lists!$C:$C)-1,1)</definedName>
-    <definedName name="adv">OFFSET(Lists!$D$2,0,0,COUNTA(Lists!$D:$D)-1,1)</definedName>
-    <definedName name="col">OFFSET(Lists!$E$2,0,0,COUNTA(Lists!$E:$E)-1,1)</definedName>
-    <definedName name="edi">OFFSET(Lists!$F$2,0,0,COUNTA(Lists!$F:$F)-1,1)</definedName>
-    <definedName name="inv">OFFSET(Lists!$G$2,0,0,COUNTA(Lists!$G:$G)-1,1)</definedName>
-    <definedName name="eph">OFFSET(Lists!$H$2,0,0,COUNTA(Lists!$H:$H)-1,1)</definedName>
-    <definedName name="desc_adv">OFFSET(Lists!$I$2,0,0,COUNTA(Lists!$I:$I)-1,1)</definedName>
-    <definedName name="desc_col">OFFSET(Lists!$J$2,0,0,COUNTA(Lists!$J:$J)-1,1)</definedName>
-    <definedName name="fragrance">OFFSET(Lists!$K$2,0,0,COUNTA(Lists!$K:$K)-1,1)</definedName>
-    <definedName name="jeans">OFFSET(Lists!$L$2,0,0,COUNTA(Lists!$L:$L)-1,1)</definedName>
-    <definedName name="underwear">OFFSET(Lists!$M$2,0,0,COUNTA(Lists!$M:$M)-1,1)</definedName>
-    <definedName name="eyewear">OFFSET(Lists!$N$2,0,0,COUNTA(Lists!$N:$N)-1,1)</definedName>
-    <definedName name="denim">OFFSET(Lists!$O$2,0,0,COUNTA(Lists!$O:$O)-1,1)</definedName>
-    <definedName name="accessories">OFFSET(Lists!$P$2,0,0,COUNTA(Lists!$P:$P)-1,1)</definedName>
-    <definedName name="shoes">OFFSET(Lists!$Q$2,0,0,COUNTA(Lists!$Q:$Q)-1,1)</definedName>
-    <definedName name="rtw">OFFSET(Lists!$R$2,0,0,COUNTA(Lists!$R:$R)-1,1)</definedName>
-    <definedName name="photographers">OFFSET(Lists!$S$2,0,0,COUNTA(Lists!$S:$S)-1,1)</definedName>
-    <definedName name="directors">OFFSET(Lists!$T$2,0,0,COUNTA(Lists!$T:$T)-1,1)</definedName>
-    <definedName name="models">OFFSET(Lists!$U$2,0,0,COUNTA(Lists!$U:$U)-1,1)</definedName>
-    <definedName name="stylists">OFFSET(Lists!$V$2,0,0,COUNTA(Lists!$V:$V)-1,1)</definedName>
-    <definedName name="hair_list">OFFSET(Lists!$W$2,0,0,COUNTA(Lists!$W:$W)-1,1)</definedName>
-    <definedName name="makeup_list">OFFSET(Lists!$X$2,0,0,COUNTA(Lists!$X:$X)-1,1)</definedName>
-    <definedName name="art_directors">OFFSET(Lists!$Y$2,0,0,COUNTA(Lists!$Y:$Y)-1,1)</definedName>
-    <definedName name="creative_directors">OFFSET(Lists!$Z$2,0,0,COUNTA(Lists!$Z:$Z)-1,1)</definedName>
-    <definedName name="set_designers">OFFSET(Lists!$AA$2,0,0,COUNTA(Lists!$AA:$AA)-1,1)</definedName>
-    <definedName name="casting_directors">OFFSET(Lists!$AB$2,0,0,COUNTA(Lists!$AB:$AB)-1,1)</definedName>
-    <definedName name="production_companies">OFFSET(Lists!$AC$2,0,0,COUNTA(Lists!$AC:$AC)-1,1)</definedName>
-    <definedName name="agencies">OFFSET(Lists!$AD$2,0,0,COUNTA(Lists!$AD:$AD)-1,1)</definedName>
-    <definedName name="publications">OFFSET(Lists!$AE$2,0,0,COUNTA(Lists!$AE:$AE)-1,1)</definedName>
+    <definedName name="years">tbl_years[years]</definedName>
+    <definedName name="seasons">tbl_seasons[seasons]</definedName>
+    <definedName name="categories">tbl_categories[categories]</definedName>
+    <definedName name="adv">tbl_adv[adv]</definedName>
+    <definedName name="col">tbl_col[col]</definedName>
+    <definedName name="edi">tbl_edi[edi]</definedName>
+    <definedName name="inv">tbl_inv[inv]</definedName>
+    <definedName name="eph">tbl_eph[eph]</definedName>
+    <definedName name="desc_adv">tbl_desc_adv[desc_adv]</definedName>
+    <definedName name="desc_col">tbl_desc_col[desc_col]</definedName>
+    <definedName name="fragrance">tbl_fragrance[fragrance]</definedName>
+    <definedName name="jeans">tbl_jeans[jeans]</definedName>
+    <definedName name="underwear">tbl_underwear[underwear]</definedName>
+    <definedName name="eyewear">tbl_eyewear[eyewear]</definedName>
+    <definedName name="denim">tbl_denim[denim]</definedName>
+    <definedName name="accessories">tbl_accessories[accessories]</definedName>
+    <definedName name="shoes">tbl_shoes[shoes]</definedName>
+    <definedName name="rtw">tbl_rtw[rtw]</definedName>
+    <definedName name="photographers">tbl_photographers[photographers]</definedName>
+    <definedName name="directors">tbl_directors[directors]</definedName>
+    <definedName name="models">tbl_models[models]</definedName>
+    <definedName name="stylists">tbl_stylists[stylists]</definedName>
+    <definedName name="hair_list">tbl_hair_list[hair_list]</definedName>
+    <definedName name="makeup_list">tbl_makeup_list[makeup_list]</definedName>
+    <definedName name="art_directors">tbl_art_directors[art_directors]</definedName>
+    <definedName name="creative_directors">tbl_creative_directors[creative_directors]</definedName>
+    <definedName name="set_designers">tbl_set_designers[set_designers]</definedName>
+    <definedName name="casting_directors">tbl_casting_directors[casting_directors]</definedName>
+    <definedName name="production_companies">tbl_production_companies[production_companies]</definedName>
+    <definedName name="agencies">tbl_agencies[agencies]</definedName>
+    <definedName name="publications">tbl_publications[publications]</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -155,6 +155,316 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_years" displayName="tbl_years" ref="A1:A60" headerRowCount="1">
+  <autoFilter ref="A1:A60"/>
+  <tableColumns count="1">
+    <tableColumn id="1" name="years"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tbl_desc_col" displayName="tbl_desc_col" ref="J1:J4" headerRowCount="1">
+  <autoFilter ref="J1:J4"/>
+  <tableColumns count="1">
+    <tableColumn id="10" name="desc_col"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tbl_fragrance" displayName="tbl_fragrance" ref="K1:K13" headerRowCount="1">
+  <autoFilter ref="K1:K13"/>
+  <tableColumns count="1">
+    <tableColumn id="11" name="fragrance"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tbl_jeans" displayName="tbl_jeans" ref="L1:L5" headerRowCount="1">
+  <autoFilter ref="L1:L5"/>
+  <tableColumns count="1">
+    <tableColumn id="12" name="jeans"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tbl_underwear" displayName="tbl_underwear" ref="M1:M4" headerRowCount="1">
+  <autoFilter ref="M1:M4"/>
+  <tableColumns count="1">
+    <tableColumn id="13" name="underwear"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="tbl_eyewear" displayName="tbl_eyewear" ref="N1:N2" headerRowCount="1">
+  <autoFilter ref="N1:N2"/>
+  <tableColumns count="1">
+    <tableColumn id="14" name="eyewear"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="tbl_denim" displayName="tbl_denim" ref="O1:O2" headerRowCount="1">
+  <autoFilter ref="O1:O2"/>
+  <tableColumns count="1">
+    <tableColumn id="15" name="denim"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="tbl_accessories" displayName="tbl_accessories" ref="P1:P2" headerRowCount="1">
+  <autoFilter ref="P1:P2"/>
+  <tableColumns count="1">
+    <tableColumn id="16" name="accessories"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="tbl_shoes" displayName="tbl_shoes" ref="Q1:Q2" headerRowCount="1">
+  <autoFilter ref="Q1:Q2"/>
+  <tableColumns count="1">
+    <tableColumn id="17" name="shoes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="tbl_rtw" displayName="tbl_rtw" ref="R1:R2" headerRowCount="1">
+  <autoFilter ref="R1:R2"/>
+  <tableColumns count="1">
+    <tableColumn id="18" name="rtw"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="tbl_photographers" displayName="tbl_photographers" ref="S1:S31" headerRowCount="1">
+  <autoFilter ref="S1:S31"/>
+  <tableColumns count="1">
+    <tableColumn id="19" name="photographers"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_seasons" displayName="tbl_seasons" ref="B1:B7" headerRowCount="1">
+  <autoFilter ref="B1:B7"/>
+  <tableColumns count="1">
+    <tableColumn id="2" name="seasons"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="tbl_directors" displayName="tbl_directors" ref="T1:T16" headerRowCount="1">
+  <autoFilter ref="T1:T16"/>
+  <tableColumns count="1">
+    <tableColumn id="20" name="directors"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="tbl_models" displayName="tbl_models" ref="U1:U27" headerRowCount="1">
+  <autoFilter ref="U1:U27"/>
+  <tableColumns count="1">
+    <tableColumn id="21" name="models"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="tbl_stylists" displayName="tbl_stylists" ref="V1:V13" headerRowCount="1">
+  <autoFilter ref="V1:V13"/>
+  <tableColumns count="1">
+    <tableColumn id="22" name="stylists"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="tbl_hair_list" displayName="tbl_hair_list" ref="W1:W10" headerRowCount="1">
+  <autoFilter ref="W1:W10"/>
+  <tableColumns count="1">
+    <tableColumn id="23" name="hair_list"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="tbl_makeup_list" displayName="tbl_makeup_list" ref="X1:X11" headerRowCount="1">
+  <autoFilter ref="X1:X11"/>
+  <tableColumns count="1">
+    <tableColumn id="24" name="makeup_list"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="tbl_art_directors" displayName="tbl_art_directors" ref="Y1:Y6" headerRowCount="1">
+  <autoFilter ref="Y1:Y6"/>
+  <tableColumns count="1">
+    <tableColumn id="25" name="art_directors"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="tbl_creative_directors" displayName="tbl_creative_directors" ref="Z1:Z8" headerRowCount="1">
+  <autoFilter ref="Z1:Z8"/>
+  <tableColumns count="1">
+    <tableColumn id="26" name="creative_directors"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="tbl_set_designers" displayName="tbl_set_designers" ref="AA1:AA6" headerRowCount="1">
+  <autoFilter ref="AA1:AA6"/>
+  <tableColumns count="1">
+    <tableColumn id="27" name="set_designers"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="tbl_casting_directors" displayName="tbl_casting_directors" ref="AB1:AB6" headerRowCount="1">
+  <autoFilter ref="AB1:AB6"/>
+  <tableColumns count="1">
+    <tableColumn id="28" name="casting_directors"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="tbl_production_companies" displayName="tbl_production_companies" ref="AC1:AC7" headerRowCount="1">
+  <autoFilter ref="AC1:AC7"/>
+  <tableColumns count="1">
+    <tableColumn id="29" name="production_companies"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tbl_categories" displayName="tbl_categories" ref="C1:C6" headerRowCount="1">
+  <autoFilter ref="C1:C6"/>
+  <tableColumns count="1">
+    <tableColumn id="3" name="categories"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="tbl_agencies" displayName="tbl_agencies" ref="AD1:AD7" headerRowCount="1">
+  <autoFilter ref="AD1:AD7"/>
+  <tableColumns count="1">
+    <tableColumn id="30" name="agencies"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="tbl_publications" displayName="tbl_publications" ref="AE1:AE17" headerRowCount="1">
+  <autoFilter ref="AE1:AE17"/>
+  <tableColumns count="1">
+    <tableColumn id="31" name="publications"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbl_adv" displayName="tbl_adv" ref="D1:D5" headerRowCount="1">
+  <autoFilter ref="D1:D5"/>
+  <tableColumns count="1">
+    <tableColumn id="4" name="adv"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tbl_col" displayName="tbl_col" ref="E1:E6" headerRowCount="1">
+  <autoFilter ref="E1:E6"/>
+  <tableColumns count="1">
+    <tableColumn id="5" name="col"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tbl_edi" displayName="tbl_edi" ref="F1:F11" headerRowCount="1">
+  <autoFilter ref="F1:F11"/>
+  <tableColumns count="1">
+    <tableColumn id="6" name="edi"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tbl_inv" displayName="tbl_inv" ref="G1:G3" headerRowCount="1">
+  <autoFilter ref="G1:G3"/>
+  <tableColumns count="1">
+    <tableColumn id="7" name="inv"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tbl_eph" displayName="tbl_eph" ref="H1:H5" headerRowCount="1">
+  <autoFilter ref="H1:H5"/>
+  <tableColumns count="1">
+    <tableColumn id="8" name="eph"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tbl_desc_adv" displayName="tbl_desc_adv" ref="I1:I9" headerRowCount="1">
+  <autoFilter ref="I1:I9"/>
+  <tableColumns count="1">
+    <tableColumn id="9" name="desc_adv"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2245,5 +2555,38 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="31">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId20"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId21"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId22"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId25"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId26"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId27"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId28"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId30"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId31"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove source_url column from archive index
https://claude.ai/code/session_01LG1wPERtMFPnjz7WXpbQZ4
</commit_message>
<xml_diff>
--- a/archive_index.xlsx
+++ b/archive_index.xlsx
@@ -2,48 +2,47 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Archive" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Lists" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="years">tbl_years[years]</definedName>
-    <definedName name="seasons">tbl_seasons[seasons]</definedName>
+    <definedName name="accessories">tbl_accessories[accessories]</definedName>
+    <definedName name="adv">tbl_adv[adv]</definedName>
+    <definedName name="agencies">tbl_agencies[agencies]</definedName>
+    <definedName name="art_directors">tbl_art_directors[art_directors]</definedName>
+    <definedName name="casting_directors">tbl_casting_directors[casting_directors]</definedName>
     <definedName name="categories">tbl_categories[categories]</definedName>
-    <definedName name="adv">tbl_adv[adv]</definedName>
     <definedName name="col">tbl_col[col]</definedName>
-    <definedName name="edi">tbl_edi[edi]</definedName>
-    <definedName name="inv">tbl_inv[inv]</definedName>
-    <definedName name="eph">tbl_eph[eph]</definedName>
+    <definedName name="creative_directors">tbl_creative_directors[creative_directors]</definedName>
+    <definedName name="denim">tbl_denim[denim]</definedName>
     <definedName name="desc_adv">tbl_desc_adv[desc_adv]</definedName>
     <definedName name="desc_col">tbl_desc_col[desc_col]</definedName>
+    <definedName name="directors">tbl_directors[directors]</definedName>
+    <definedName name="edi">tbl_edi[edi]</definedName>
+    <definedName name="eph">tbl_eph[eph]</definedName>
+    <definedName name="eyewear">tbl_eyewear[eyewear]</definedName>
     <definedName name="fragrance">tbl_fragrance[fragrance]</definedName>
+    <definedName name="hair_list">tbl_hair_list[hair_list]</definedName>
+    <definedName name="inv">tbl_inv[inv]</definedName>
     <definedName name="jeans">tbl_jeans[jeans]</definedName>
+    <definedName name="makeup_list">tbl_makeup_list[makeup_list]</definedName>
+    <definedName name="models">tbl_models[models]</definedName>
+    <definedName name="photographers">tbl_photographers[photographers]</definedName>
+    <definedName name="production_companies">tbl_production_companies[production_companies]</definedName>
+    <definedName name="publications">tbl_publications[publications]</definedName>
+    <definedName name="rtw">tbl_rtw[rtw]</definedName>
+    <definedName name="seasons">tbl_seasons[seasons]</definedName>
+    <definedName name="set_designers">tbl_set_designers[set_designers]</definedName>
+    <definedName name="shoes">tbl_shoes[shoes]</definedName>
+    <definedName name="stylists">tbl_stylists[stylists]</definedName>
     <definedName name="underwear">tbl_underwear[underwear]</definedName>
-    <definedName name="eyewear">tbl_eyewear[eyewear]</definedName>
-    <definedName name="denim">tbl_denim[denim]</definedName>
-    <definedName name="accessories">tbl_accessories[accessories]</definedName>
-    <definedName name="shoes">tbl_shoes[shoes]</definedName>
-    <definedName name="rtw">tbl_rtw[rtw]</definedName>
-    <definedName name="photographers">tbl_photographers[photographers]</definedName>
-    <definedName name="directors">tbl_directors[directors]</definedName>
-    <definedName name="models">tbl_models[models]</definedName>
-    <definedName name="stylists">tbl_stylists[stylists]</definedName>
-    <definedName name="hair_list">tbl_hair_list[hair_list]</definedName>
-    <definedName name="makeup_list">tbl_makeup_list[makeup_list]</definedName>
-    <definedName name="art_directors">tbl_art_directors[art_directors]</definedName>
-    <definedName name="creative_directors">tbl_creative_directors[creative_directors]</definedName>
-    <definedName name="set_designers">tbl_set_designers[set_designers]</definedName>
-    <definedName name="casting_directors">tbl_casting_directors[casting_directors]</definedName>
-    <definedName name="production_companies">tbl_production_companies[production_companies]</definedName>
-    <definedName name="agencies">tbl_agencies[agencies]</definedName>
-    <definedName name="publications">tbl_publications[publications]</definedName>
+    <definedName name="years">tbl_years[years]</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -79,11 +78,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -163,7 +163,7 @@
   <tableColumns count="1">
     <tableColumn id="1" name="years"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -173,7 +173,7 @@
   <tableColumns count="1">
     <tableColumn id="10" name="desc_col"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -183,7 +183,7 @@
   <tableColumns count="1">
     <tableColumn id="11" name="fragrance"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -193,7 +193,7 @@
   <tableColumns count="1">
     <tableColumn id="12" name="jeans"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -203,7 +203,7 @@
   <tableColumns count="1">
     <tableColumn id="13" name="underwear"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -213,7 +213,7 @@
   <tableColumns count="1">
     <tableColumn id="14" name="eyewear"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -223,7 +223,7 @@
   <tableColumns count="1">
     <tableColumn id="15" name="denim"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -233,7 +233,7 @@
   <tableColumns count="1">
     <tableColumn id="16" name="accessories"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -243,7 +243,7 @@
   <tableColumns count="1">
     <tableColumn id="17" name="shoes"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -253,7 +253,7 @@
   <tableColumns count="1">
     <tableColumn id="18" name="rtw"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -263,7 +263,7 @@
   <tableColumns count="1">
     <tableColumn id="19" name="photographers"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -273,7 +273,7 @@
   <tableColumns count="1">
     <tableColumn id="2" name="seasons"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -283,7 +283,7 @@
   <tableColumns count="1">
     <tableColumn id="20" name="directors"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -293,7 +293,7 @@
   <tableColumns count="1">
     <tableColumn id="21" name="models"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -303,7 +303,7 @@
   <tableColumns count="1">
     <tableColumn id="22" name="stylists"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -313,7 +313,7 @@
   <tableColumns count="1">
     <tableColumn id="23" name="hair_list"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -323,7 +323,7 @@
   <tableColumns count="1">
     <tableColumn id="24" name="makeup_list"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -333,7 +333,7 @@
   <tableColumns count="1">
     <tableColumn id="25" name="art_directors"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -343,7 +343,7 @@
   <tableColumns count="1">
     <tableColumn id="26" name="creative_directors"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -353,7 +353,7 @@
   <tableColumns count="1">
     <tableColumn id="27" name="set_designers"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -363,7 +363,7 @@
   <tableColumns count="1">
     <tableColumn id="28" name="casting_directors"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -373,7 +373,7 @@
   <tableColumns count="1">
     <tableColumn id="29" name="production_companies"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -383,7 +383,7 @@
   <tableColumns count="1">
     <tableColumn id="3" name="categories"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -393,7 +393,7 @@
   <tableColumns count="1">
     <tableColumn id="30" name="agencies"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -403,7 +403,7 @@
   <tableColumns count="1">
     <tableColumn id="31" name="publications"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -413,7 +413,7 @@
   <tableColumns count="1">
     <tableColumn id="4" name="adv"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -423,7 +423,7 @@
   <tableColumns count="1">
     <tableColumn id="5" name="col"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -433,7 +433,7 @@
   <tableColumns count="1">
     <tableColumn id="6" name="edi"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -443,7 +443,7 @@
   <tableColumns count="1">
     <tableColumn id="7" name="inv"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -453,17 +453,17 @@
   <tableColumns count="1">
     <tableColumn id="8" name="eph"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tbl_desc_adv" displayName="tbl_desc_adv" ref="I1:I9" headerRowCount="1">
-  <autoFilter ref="I1:I9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tbl_desc_adv" displayName="tbl_desc_adv" ref="I1:I10" headerRowCount="1">
+  <autoFilter ref="I1:I10"/>
   <tableColumns count="1">
     <tableColumn id="9" name="desc_adv"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -756,34 +756,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:X1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="30" customWidth="1" min="24" max="24"/>
-    <col width="24" customWidth="1" min="25" max="25"/>
+    <col width="38" customWidth="1" style="1" min="1" max="1"/>
+    <col width="6" customWidth="1" style="1" min="2" max="2"/>
+    <col width="8" customWidth="1" style="1" min="3" max="4"/>
+    <col width="12" customWidth="1" style="1" min="5" max="5"/>
+    <col width="14" customWidth="1" style="1" min="6" max="6"/>
+    <col width="20" customWidth="1" style="1" min="7" max="7"/>
+    <col width="22" customWidth="1" style="1" min="8" max="8"/>
+    <col width="18" customWidth="1" style="1" min="9" max="9"/>
+    <col width="16" customWidth="1" style="1" min="10" max="10"/>
+    <col width="22" customWidth="1" style="1" min="11" max="11"/>
+    <col width="20" customWidth="1" style="1" min="12" max="12"/>
+    <col width="22" customWidth="1" style="1" min="13" max="13"/>
+    <col width="18" customWidth="1" style="1" min="14" max="14"/>
+    <col width="20" customWidth="1" style="1" min="15" max="15"/>
+    <col width="18" customWidth="1" style="1" min="16" max="18"/>
+    <col width="20" customWidth="1" style="1" min="19" max="19"/>
+    <col width="16" customWidth="1" style="1" min="20" max="20"/>
+    <col width="18" customWidth="1" style="1" min="21" max="21"/>
+    <col width="14" customWidth="1" style="1" min="22" max="22"/>
+    <col width="18" customWidth="1" style="1" min="23" max="23"/>
+    <col width="30" customWidth="1" style="1" min="24" max="24"/>
+    <col width="24" customWidth="1" style="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -904,11 +901,6 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>source_url</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
           <t>notes</t>
         </is>
       </c>
@@ -916,61 +908,61 @@
   </sheetData>
   <dataValidations count="19">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=years</formula1>
+      <formula1>years</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>=seasons</formula1>
+      <formula1>seasons</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>=categories</formula1>
+      <formula1>categories</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=photographers</formula1>
+      <formula1>photographers</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=directors</formula1>
+      <formula1>directors</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=models</formula1>
+      <formula1>models</formula1>
     </dataValidation>
     <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=stylists</formula1>
+      <formula1>stylists</formula1>
     </dataValidation>
     <dataValidation sqref="P2:P1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=hair_list</formula1>
+      <formula1>hair_list</formula1>
     </dataValidation>
     <dataValidation sqref="Q2:Q1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=makeup_list</formula1>
+      <formula1>makeup_list</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=art_directors</formula1>
+      <formula1>art_directors</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=creative_directors</formula1>
+      <formula1>creative_directors</formula1>
     </dataValidation>
     <dataValidation sqref="R2:R1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=set_designers</formula1>
+      <formula1>set_designers</formula1>
     </dataValidation>
     <dataValidation sqref="S2:S1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=casting_directors</formula1>
+      <formula1>casting_directors</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=production_companies</formula1>
+      <formula1>production_companies</formula1>
     </dataValidation>
     <dataValidation sqref="T2:T1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=agencies</formula1>
+      <formula1>agencies</formula1>
     </dataValidation>
     <dataValidation sqref="U2:U1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=publications</formula1>
+      <formula1>publications</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=INDIRECT($D2)</formula1>
+      <formula1>INDIRECT($D2)</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=INDIRECT("desc_"&amp;$D2)</formula1>
+      <formula1>INDIRECT("desc_"&amp;$D2)</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=INDIRECT(SUBSTITUTE($F2," ","_"))</formula1>
+      <formula1>INDIRECT(SUBSTITUTE($F2," ","_"))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -984,7 +976,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AE60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1434,7 +1426,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>aw</t>
+          <t>cruise</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1559,7 +1551,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>cruise</t>
+          <t>pre-fall</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1674,7 +1666,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>pre-fall</t>
+          <t>resort</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1772,11 +1764,6 @@
       <c r="A7" t="n">
         <v>1973</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>resort</t>
-        </is>
-      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>dazed</t>
@@ -1965,6 +1952,11 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>numero</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>watches</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">

</xml_diff>

<commit_message>
Replace adv lines with CK product lines and expand campaign lists
https://claude.ai/code/session_01LG1wPERtMFPnjz7WXpbQZ4
</commit_message>
<xml_diff>
--- a/archive_index.xlsx
+++ b/archive_index.xlsx
@@ -2,47 +2,44 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Archive" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Lists" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="accessories">tbl_accessories[accessories]</definedName>
+    <definedName name="years">tbl_years[years]</definedName>
+    <definedName name="seasons">tbl_seasons[seasons]</definedName>
+    <definedName name="categories">tbl_categories[categories]</definedName>
     <definedName name="adv">tbl_adv[adv]</definedName>
-    <definedName name="agencies">tbl_agencies[agencies]</definedName>
-    <definedName name="art_directors">tbl_art_directors[art_directors]</definedName>
-    <definedName name="casting_directors">tbl_casting_directors[casting_directors]</definedName>
-    <definedName name="categories">tbl_categories[categories]</definedName>
     <definedName name="col">tbl_col[col]</definedName>
-    <definedName name="creative_directors">tbl_creative_directors[creative_directors]</definedName>
-    <definedName name="denim">tbl_denim[denim]</definedName>
+    <definedName name="edi">tbl_edi[edi]</definedName>
+    <definedName name="inv">tbl_inv[inv]</definedName>
+    <definedName name="eph">tbl_eph[eph]</definedName>
     <definedName name="desc_adv">tbl_desc_adv[desc_adv]</definedName>
     <definedName name="desc_col">tbl_desc_col[desc_col]</definedName>
-    <definedName name="directors">tbl_directors[directors]</definedName>
-    <definedName name="edi">tbl_edi[edi]</definedName>
-    <definedName name="eph">tbl_eph[eph]</definedName>
+    <definedName name="jeans">tbl_jeans[jeans]</definedName>
+    <definedName name="underwear">tbl_underwear[underwear]</definedName>
     <definedName name="eyewear">tbl_eyewear[eyewear]</definedName>
     <definedName name="fragrance">tbl_fragrance[fragrance]</definedName>
+    <definedName name="photographers">tbl_photographers[photographers]</definedName>
+    <definedName name="directors">tbl_directors[directors]</definedName>
+    <definedName name="models">tbl_models[models]</definedName>
+    <definedName name="stylists">tbl_stylists[stylists]</definedName>
     <definedName name="hair_list">tbl_hair_list[hair_list]</definedName>
-    <definedName name="inv">tbl_inv[inv]</definedName>
-    <definedName name="jeans">tbl_jeans[jeans]</definedName>
     <definedName name="makeup_list">tbl_makeup_list[makeup_list]</definedName>
-    <definedName name="models">tbl_models[models]</definedName>
-    <definedName name="photographers">tbl_photographers[photographers]</definedName>
+    <definedName name="art_directors">tbl_art_directors[art_directors]</definedName>
+    <definedName name="creative_directors">tbl_creative_directors[creative_directors]</definedName>
+    <definedName name="set_designers">tbl_set_designers[set_designers]</definedName>
+    <definedName name="casting_directors">tbl_casting_directors[casting_directors]</definedName>
     <definedName name="production_companies">tbl_production_companies[production_companies]</definedName>
+    <definedName name="agencies">tbl_agencies[agencies]</definedName>
     <definedName name="publications">tbl_publications[publications]</definedName>
-    <definedName name="rtw">tbl_rtw[rtw]</definedName>
-    <definedName name="seasons">tbl_seasons[seasons]</definedName>
-    <definedName name="set_designers">tbl_set_designers[set_designers]</definedName>
-    <definedName name="shoes">tbl_shoes[shoes]</definedName>
-    <definedName name="stylists">tbl_stylists[stylists]</definedName>
-    <definedName name="underwear">tbl_underwear[underwear]</definedName>
-    <definedName name="years">tbl_years[years]</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -78,12 +75,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -163,7 +159,7 @@
   <tableColumns count="1">
     <tableColumn id="1" name="years"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -173,207 +169,187 @@
   <tableColumns count="1">
     <tableColumn id="10" name="desc_col"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tbl_fragrance" displayName="tbl_fragrance" ref="K1:K13" headerRowCount="1">
-  <autoFilter ref="K1:K13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tbl_jeans" displayName="tbl_jeans" ref="K1:K11" headerRowCount="1">
+  <autoFilter ref="K1:K11"/>
   <tableColumns count="1">
-    <tableColumn id="11" name="fragrance"/>
+    <tableColumn id="11" name="jeans"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tbl_jeans" displayName="tbl_jeans" ref="L1:L5" headerRowCount="1">
-  <autoFilter ref="L1:L5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tbl_underwear" displayName="tbl_underwear" ref="L1:L12" headerRowCount="1">
+  <autoFilter ref="L1:L12"/>
   <tableColumns count="1">
-    <tableColumn id="12" name="jeans"/>
+    <tableColumn id="12" name="underwear"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tbl_underwear" displayName="tbl_underwear" ref="M1:M4" headerRowCount="1">
-  <autoFilter ref="M1:M4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tbl_eyewear" displayName="tbl_eyewear" ref="M1:M2" headerRowCount="1">
+  <autoFilter ref="M1:M2"/>
   <tableColumns count="1">
-    <tableColumn id="13" name="underwear"/>
+    <tableColumn id="13" name="eyewear"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="tbl_eyewear" displayName="tbl_eyewear" ref="N1:N2" headerRowCount="1">
-  <autoFilter ref="N1:N2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="tbl_fragrance" displayName="tbl_fragrance" ref="N1:N34" headerRowCount="1">
+  <autoFilter ref="N1:N34"/>
   <tableColumns count="1">
-    <tableColumn id="14" name="eyewear"/>
+    <tableColumn id="14" name="fragrance"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="tbl_denim" displayName="tbl_denim" ref="O1:O2" headerRowCount="1">
-  <autoFilter ref="O1:O2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="tbl_photographers" displayName="tbl_photographers" ref="O1:O31" headerRowCount="1">
+  <autoFilter ref="O1:O31"/>
   <tableColumns count="1">
-    <tableColumn id="15" name="denim"/>
+    <tableColumn id="15" name="photographers"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="tbl_accessories" displayName="tbl_accessories" ref="P1:P2" headerRowCount="1">
-  <autoFilter ref="P1:P2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="tbl_directors" displayName="tbl_directors" ref="P1:P16" headerRowCount="1">
+  <autoFilter ref="P1:P16"/>
   <tableColumns count="1">
-    <tableColumn id="16" name="accessories"/>
+    <tableColumn id="16" name="directors"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="tbl_shoes" displayName="tbl_shoes" ref="Q1:Q2" headerRowCount="1">
-  <autoFilter ref="Q1:Q2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="tbl_models" displayName="tbl_models" ref="Q1:Q27" headerRowCount="1">
+  <autoFilter ref="Q1:Q27"/>
   <tableColumns count="1">
-    <tableColumn id="17" name="shoes"/>
+    <tableColumn id="17" name="models"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="tbl_rtw" displayName="tbl_rtw" ref="R1:R2" headerRowCount="1">
-  <autoFilter ref="R1:R2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="tbl_stylists" displayName="tbl_stylists" ref="R1:R13" headerRowCount="1">
+  <autoFilter ref="R1:R13"/>
   <tableColumns count="1">
-    <tableColumn id="18" name="rtw"/>
+    <tableColumn id="18" name="stylists"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="tbl_photographers" displayName="tbl_photographers" ref="S1:S31" headerRowCount="1">
-  <autoFilter ref="S1:S31"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="tbl_hair_list" displayName="tbl_hair_list" ref="S1:S10" headerRowCount="1">
+  <autoFilter ref="S1:S10"/>
   <tableColumns count="1">
-    <tableColumn id="19" name="photographers"/>
+    <tableColumn id="19" name="hair_list"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_seasons" displayName="tbl_seasons" ref="B1:B7" headerRowCount="1">
-  <autoFilter ref="B1:B7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_seasons" displayName="tbl_seasons" ref="B1:B6" headerRowCount="1">
+  <autoFilter ref="B1:B6"/>
   <tableColumns count="1">
     <tableColumn id="2" name="seasons"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="tbl_directors" displayName="tbl_directors" ref="T1:T16" headerRowCount="1">
-  <autoFilter ref="T1:T16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="tbl_makeup_list" displayName="tbl_makeup_list" ref="T1:T11" headerRowCount="1">
+  <autoFilter ref="T1:T11"/>
   <tableColumns count="1">
-    <tableColumn id="20" name="directors"/>
+    <tableColumn id="20" name="makeup_list"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="tbl_models" displayName="tbl_models" ref="U1:U27" headerRowCount="1">
-  <autoFilter ref="U1:U27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="tbl_art_directors" displayName="tbl_art_directors" ref="U1:U6" headerRowCount="1">
+  <autoFilter ref="U1:U6"/>
   <tableColumns count="1">
-    <tableColumn id="21" name="models"/>
+    <tableColumn id="21" name="art_directors"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="tbl_stylists" displayName="tbl_stylists" ref="V1:V13" headerRowCount="1">
-  <autoFilter ref="V1:V13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="tbl_creative_directors" displayName="tbl_creative_directors" ref="V1:V8" headerRowCount="1">
+  <autoFilter ref="V1:V8"/>
   <tableColumns count="1">
-    <tableColumn id="22" name="stylists"/>
+    <tableColumn id="22" name="creative_directors"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="tbl_hair_list" displayName="tbl_hair_list" ref="W1:W10" headerRowCount="1">
-  <autoFilter ref="W1:W10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="tbl_set_designers" displayName="tbl_set_designers" ref="W1:W6" headerRowCount="1">
+  <autoFilter ref="W1:W6"/>
   <tableColumns count="1">
-    <tableColumn id="23" name="hair_list"/>
+    <tableColumn id="23" name="set_designers"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="tbl_makeup_list" displayName="tbl_makeup_list" ref="X1:X11" headerRowCount="1">
-  <autoFilter ref="X1:X11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="tbl_casting_directors" displayName="tbl_casting_directors" ref="X1:X6" headerRowCount="1">
+  <autoFilter ref="X1:X6"/>
   <tableColumns count="1">
-    <tableColumn id="24" name="makeup_list"/>
+    <tableColumn id="24" name="casting_directors"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="tbl_art_directors" displayName="tbl_art_directors" ref="Y1:Y6" headerRowCount="1">
-  <autoFilter ref="Y1:Y6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="tbl_production_companies" displayName="tbl_production_companies" ref="Y1:Y7" headerRowCount="1">
+  <autoFilter ref="Y1:Y7"/>
   <tableColumns count="1">
-    <tableColumn id="25" name="art_directors"/>
+    <tableColumn id="25" name="production_companies"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="tbl_creative_directors" displayName="tbl_creative_directors" ref="Z1:Z8" headerRowCount="1">
-  <autoFilter ref="Z1:Z8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="tbl_agencies" displayName="tbl_agencies" ref="Z1:Z7" headerRowCount="1">
+  <autoFilter ref="Z1:Z7"/>
   <tableColumns count="1">
-    <tableColumn id="26" name="creative_directors"/>
+    <tableColumn id="26" name="agencies"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="tbl_set_designers" displayName="tbl_set_designers" ref="AA1:AA6" headerRowCount="1">
-  <autoFilter ref="AA1:AA6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="tbl_publications" displayName="tbl_publications" ref="AA1:AA17" headerRowCount="1">
+  <autoFilter ref="AA1:AA17"/>
   <tableColumns count="1">
-    <tableColumn id="27" name="set_designers"/>
+    <tableColumn id="27" name="publications"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="tbl_casting_directors" displayName="tbl_casting_directors" ref="AB1:AB6" headerRowCount="1">
-  <autoFilter ref="AB1:AB6"/>
-  <tableColumns count="1">
-    <tableColumn id="28" name="casting_directors"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="tbl_production_companies" displayName="tbl_production_companies" ref="AC1:AC7" headerRowCount="1">
-  <autoFilter ref="AC1:AC7"/>
-  <tableColumns count="1">
-    <tableColumn id="29" name="production_companies"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -383,27 +359,7 @@
   <tableColumns count="1">
     <tableColumn id="3" name="categories"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="tbl_agencies" displayName="tbl_agencies" ref="AD1:AD7" headerRowCount="1">
-  <autoFilter ref="AD1:AD7"/>
-  <tableColumns count="1">
-    <tableColumn id="30" name="agencies"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="tbl_publications" displayName="tbl_publications" ref="AE1:AE17" headerRowCount="1">
-  <autoFilter ref="AE1:AE17"/>
-  <tableColumns count="1">
-    <tableColumn id="31" name="publications"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -413,7 +369,7 @@
   <tableColumns count="1">
     <tableColumn id="4" name="adv"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -423,7 +379,7 @@
   <tableColumns count="1">
     <tableColumn id="5" name="col"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -433,7 +389,7 @@
   <tableColumns count="1">
     <tableColumn id="6" name="edi"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -443,7 +399,7 @@
   <tableColumns count="1">
     <tableColumn id="7" name="inv"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -453,17 +409,17 @@
   <tableColumns count="1">
     <tableColumn id="8" name="eph"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tbl_desc_adv" displayName="tbl_desc_adv" ref="I1:I10" headerRowCount="1">
-  <autoFilter ref="I1:I10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tbl_desc_adv" displayName="tbl_desc_adv" ref="I1:I16" headerRowCount="1">
+  <autoFilter ref="I1:I16"/>
   <tableColumns count="1">
     <tableColumn id="9" name="desc_adv"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -757,30 +713,32 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:X1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" style="1" min="1" max="1"/>
-    <col width="6" customWidth="1" style="1" min="2" max="2"/>
-    <col width="8" customWidth="1" style="1" min="3" max="4"/>
-    <col width="12" customWidth="1" style="1" min="5" max="5"/>
-    <col width="14" customWidth="1" style="1" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="7"/>
-    <col width="22" customWidth="1" style="1" min="8" max="8"/>
-    <col width="18" customWidth="1" style="1" min="9" max="9"/>
-    <col width="16" customWidth="1" style="1" min="10" max="10"/>
-    <col width="22" customWidth="1" style="1" min="11" max="11"/>
-    <col width="20" customWidth="1" style="1" min="12" max="12"/>
-    <col width="22" customWidth="1" style="1" min="13" max="13"/>
-    <col width="18" customWidth="1" style="1" min="14" max="14"/>
-    <col width="20" customWidth="1" style="1" min="15" max="15"/>
-    <col width="18" customWidth="1" style="1" min="16" max="18"/>
-    <col width="20" customWidth="1" style="1" min="19" max="19"/>
-    <col width="16" customWidth="1" style="1" min="20" max="20"/>
-    <col width="18" customWidth="1" style="1" min="21" max="21"/>
-    <col width="14" customWidth="1" style="1" min="22" max="22"/>
-    <col width="18" customWidth="1" style="1" min="23" max="23"/>
-    <col width="30" customWidth="1" style="1" min="24" max="24"/>
-    <col width="24" customWidth="1" style="1" min="25" max="25"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="24" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -908,61 +866,61 @@
   </sheetData>
   <dataValidations count="19">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>years</formula1>
+      <formula1>=years</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>seasons</formula1>
+      <formula1>=seasons</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>categories</formula1>
+      <formula1>=categories</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>photographers</formula1>
+      <formula1>=photographers</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>directors</formula1>
+      <formula1>=directors</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>models</formula1>
+      <formula1>=models</formula1>
     </dataValidation>
     <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>stylists</formula1>
+      <formula1>=stylists</formula1>
     </dataValidation>
     <dataValidation sqref="P2:P1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>hair_list</formula1>
+      <formula1>=hair_list</formula1>
     </dataValidation>
     <dataValidation sqref="Q2:Q1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>makeup_list</formula1>
+      <formula1>=makeup_list</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>art_directors</formula1>
+      <formula1>=art_directors</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>creative_directors</formula1>
+      <formula1>=creative_directors</formula1>
     </dataValidation>
     <dataValidation sqref="R2:R1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>set_designers</formula1>
+      <formula1>=set_designers</formula1>
     </dataValidation>
     <dataValidation sqref="S2:S1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>casting_directors</formula1>
+      <formula1>=casting_directors</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>production_companies</formula1>
+      <formula1>=production_companies</formula1>
     </dataValidation>
     <dataValidation sqref="T2:T1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>agencies</formula1>
+      <formula1>=agencies</formula1>
     </dataValidation>
     <dataValidation sqref="U2:U1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>publications</formula1>
+      <formula1>=publications</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>INDIRECT($D2)</formula1>
+      <formula1>=INDIRECT($D2)</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>INDIRECT("desc_"&amp;$D2)</formula1>
+      <formula1>=INDIRECT("desc_"&amp;$D2)</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>INDIRECT(SUBSTITUTE($F2," ","_"))</formula1>
+      <formula1>=INDIRECT(SUBSTITUTE($F2," ","_"))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -975,8 +933,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <dimension ref="A1:AA60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1031,105 +989,85 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>jeans</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>underwear</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>eyewear</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>fragrance</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>jeans</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>underwear</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>eyewear</t>
-        </is>
-      </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>denim</t>
+          <t>photographers</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>directors</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>shoes</t>
+          <t>models</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>rtw</t>
+          <t>stylists</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>photographers</t>
+          <t>hair_list</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>directors</t>
+          <t>makeup_list</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>models</t>
+          <t>art_directors</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>stylists</t>
+          <t>creative_directors</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>hair_list</t>
+          <t>set_designers</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>makeup_list</t>
+          <t>casting_directors</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>art_directors</t>
+          <t>production_companies</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>creative_directors</t>
+          <t>agencies</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
-        <is>
-          <t>set_designers</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>casting_directors</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>production_companies</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>agencies</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
         <is>
           <t>publications</t>
         </is>
@@ -1176,7 +1114,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>fragrance</t>
+          <t>collection</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1186,105 +1124,85 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>nothing comes between me</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>marky mark underwear</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>ck eyewear</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>obsession</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>are you wearing any</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>ck underwear</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>ck eyewear</t>
-        </is>
-      </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>ck denim</t>
+          <t>Bruce Weber</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>ck accessories</t>
+          <t>Fabien Baron</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>ck shoes</t>
+          <t>Kate Moss</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>ck rtw</t>
+          <t>Camilla Nickerson</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Bruce Weber</t>
+          <t>Garren</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
+          <t>Pat McGrath</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
           <t>Fabien Baron</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Kate Moss</t>
-        </is>
-      </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Camilla Nickerson</t>
+          <t>Calvin Klein</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Garren</t>
+          <t>Stefan Beckman</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Pat McGrath</t>
+          <t>James Scully</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Fabien Baron</t>
+          <t>Baron &amp; Baron</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Calvin Klein</t>
+          <t>Baron &amp; Baron</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
-        <is>
-          <t>Stefan Beckman</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>James Scully</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>Baron &amp; Baron</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>Baron &amp; Baron</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
         <is>
           <t>Vogue US</t>
         </is>
@@ -1331,7 +1249,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>jeans</t>
+          <t>ck white</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1341,80 +1259,80 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>eternity</t>
+          <t>marky mark</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>nothing comes between me</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>my calvins</t>
+          <t>kate moss underwear</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>obsession for men</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Steven Meisel</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>David Fincher</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Christy Turlington</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Joe McKenna</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Steven Meisel</t>
+          <t>Guido Palau</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>David Fincher</t>
+          <t>Diane Kendal</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Christy Turlington</t>
+          <t>Sam Shahid</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Joe McKenna</t>
+          <t>Raf Simons</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Guido Palau</t>
+          <t>Mary Howard</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Diane Kendal</t>
+          <t>Piergiorgio Del Moro</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Sam Shahid</t>
+          <t>CDM</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>Raf Simons</t>
+          <t>CDM</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
-        <is>
-          <t>Mary Howard</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>Piergiorgio Del Moro</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>CDM</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>CDM</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
         <is>
           <t>Vogue Italia</t>
         </is>
@@ -1456,7 +1374,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>underwear</t>
+          <t>jeans</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1466,80 +1384,80 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>ck one</t>
+          <t>kate moss obsession</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>just the way you are</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>i __ my calvins</t>
+          <t>mycalvins</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>eternity</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Richard Avedon</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Bruce Weber</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Naomi Campbell</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Karl Templer</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Richard Avedon</t>
+          <t>Sam McKnight</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Bruce Weber</t>
+          <t>Aaron de Mey</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Naomi Campbell</t>
+          <t>Tibor Kalman</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Karl Templer</t>
+          <t>Francisco Costa</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>Sam McKnight</t>
+          <t>Andy Hillman</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>Aaron de Mey</t>
+          <t>Ashley Brokaw</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>Tibor Kalman</t>
+          <t>Calvin Klein Inc.</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>Francisco Costa</t>
+          <t>Wieden+Kennedy</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
-        <is>
-          <t>Andy Hillman</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>Ashley Brokaw</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>Calvin Klein Inc.</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>Wieden+Kennedy</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
         <is>
           <t>Vogue Paris</t>
         </is>
@@ -1561,7 +1479,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>tv</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1581,80 +1499,85 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>eyewear</t>
+          <t>underwear</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>escape</t>
+          <t>heroin chic</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>ck jeans</t>
+          <t>justin bieber x lara stone</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>eternity for men</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Herb Ritts</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Sofia Coppola</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Cindy Crawford</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Marie-Amélie Sauvé</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Herb Ritts</t>
+          <t>Eugene Souleiman</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Sofia Coppola</t>
+          <t>Tom Pecheux</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Cindy Crawford</t>
+          <t>Neville Brody</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Marie-Amélie Sauvé</t>
+          <t>Italo Zucchelli</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>Eugene Souleiman</t>
+          <t>Piers Hanmer</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>Tom Pecheux</t>
+          <t>Jess Hallett</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Neville Brody</t>
+          <t>Hungry Man</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>Italo Zucchelli</t>
+          <t>Mother</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
-        <is>
-          <t>Piers Hanmer</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>Jess Hallett</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>Hungry Man</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>Mother</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
         <is>
           <t>Harper's Bazaar</t>
         </is>
@@ -1686,75 +1609,85 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>denim</t>
+          <t>performance</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>contradiction</t>
+          <t>just be</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>kendall jenner</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>escape</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Patrick Demarchelier</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Mario Sorrenti</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Linda Evangelista</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Olivier Rizzo</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Patrick Demarchelier</t>
+          <t>Christiaan Houtenbos</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Mario Sorrenti</t>
+          <t>François Nars</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Linda Evangelista</t>
+          <t>Peter Saville</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Olivier Rizzo</t>
+          <t>Kevin Carrigan</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>Christiaan Houtenbos</t>
+          <t>Jack Flanagan</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>François Nars</t>
+          <t>Anita Bitton</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Peter Saville</t>
+          <t>RSA Films</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>Kevin Carrigan</t>
+          <t>Laird+Partners</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
-        <is>
-          <t>Jack Flanagan</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>Anita Bitton</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>RSA Films</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>Laird+Partners</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
         <is>
           <t>i-D</t>
         </is>
@@ -1771,60 +1704,70 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>swimwear</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>truth</t>
+          <t>pro wash</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>i __ in mycalvins</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>escape for men</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Mario Sorrenti</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Steven Meisel</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Brooke Shields</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Alastair McKimm</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Mario Sorrenti</t>
+          <t>Didier Malige</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Steven Meisel</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Brooke Shields</t>
+          <t>Kevyn Aucoin</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Alastair McKimm</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>Didier Malige</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>Kevyn Aucoin</t>
+          <t>Pieter Mulier</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>Anonymous Content</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>Pieter Mulier</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>Anonymous Content</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
           <t>CKX</t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr">
+      <c r="AA7" t="inlineStr">
         <is>
           <t>Dazed</t>
         </is>
@@ -1841,50 +1784,60 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>shoes</t>
+          <t>golf</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>be</t>
+          <t>mycalvins</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>our now</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>ck one</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>David Sims</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Herb Ritts</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Mark Wahlberg</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Lucinda Chambers</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>David Sims</t>
+          <t>Julien d'Ys</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Herb Ritts</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Mark Wahlberg</t>
+          <t>Linda Cantello</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Lucinda Chambers</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>Julien d'Ys</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>Linda Cantello</t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
-        <is>
           <t>Veronica Leoni</t>
         </is>
       </c>
-      <c r="AE8" t="inlineStr">
+      <c r="AA8" t="inlineStr">
         <is>
           <t>Interview</t>
         </is>
@@ -1901,45 +1854,55 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>rtw</t>
+          <t>kids</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>euphoria</t>
+          <t>justin bieber</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>calvins or nothing</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>ck be</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Mert &amp; Marcus</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Spike Jonze</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Travis Fimmel</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Carlyne Cerf de Dudzeele</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Mert &amp; Marcus</t>
+          <t>Anthony Turner</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Spike Jonze</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Travis Fimmel</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>Carlyne Cerf de Dudzeele</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>Anthony Turner</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr">
-        <is>
           <t>Charlotte Tilbury</t>
         </is>
       </c>
-      <c r="AE9" t="inlineStr">
+      <c r="AA9" t="inlineStr">
         <is>
           <t>W Magazine</t>
         </is>
@@ -1956,45 +1919,55 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>watches</t>
+          <t>footwear</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>ck2</t>
+          <t>or nothing</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>jeremy allen white</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Steven Klein</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Tony Kaye</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Lara Stone</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Grace Coddington</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Steven Klein</t>
+          <t>Duffy</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Tony Kaye</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Lara Stone</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>Grace Coddington</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>Duffy</t>
-        </is>
-      </c>
-      <c r="X10" t="inlineStr">
-        <is>
           <t>Lucia Pieroni</t>
         </is>
       </c>
-      <c r="AE10" t="inlineStr">
+      <c r="AA10" t="inlineStr">
         <is>
           <t>Numéro</t>
         </is>
@@ -2009,37 +1982,52 @@
           <t>theface</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>eyewear</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>eternity moment</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
+          <t>i love my calvins</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>fka twigs or nothing</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>truth</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
         <is>
           <t>Inez &amp; Vinoodh</t>
         </is>
       </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Jonas Åkerlund</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Natalia Vodianova</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Carine Roitfeld</t>
+        </is>
+      </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Jonas Åkerlund</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Natalia Vodianova</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>Carine Roitfeld</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
           <t>Peter Philips</t>
         </is>
       </c>
-      <c r="AE11" t="inlineStr">
+      <c r="AA11" t="inlineStr">
         <is>
           <t>Self Service</t>
         </is>
@@ -2049,32 +2037,42 @@
       <c r="A12" t="n">
         <v>1978</v>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>free</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>watches jewelry</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>greta lee</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>crave</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
         <is>
           <t>Mario Testino</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>Mark Romanek</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>Jamie Dornan</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>Melanie Ward</t>
         </is>
       </c>
-      <c r="AE12" t="inlineStr">
+      <c r="AA12" t="inlineStr">
         <is>
           <t>Purple</t>
         </is>
@@ -2084,32 +2082,37 @@
       <c r="A13" t="n">
         <v>1979</v>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>ck all</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>fragrance</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>euphoria</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
         <is>
           <t>Glen Luchford</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>Floria Sigismondi</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>Gisele Bündchen</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>Tonne Goodman</t>
         </is>
       </c>
-      <c r="AE13" t="inlineStr">
+      <c r="AA13" t="inlineStr">
         <is>
           <t>Another</t>
         </is>
@@ -2119,22 +2122,32 @@
       <c r="A14" t="n">
         <v>1980</v>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>euphoria for men</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
         <is>
           <t>Craig McDean</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>Steven Klein</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>Jessica Stam</t>
         </is>
       </c>
-      <c r="AE14" t="inlineStr">
+      <c r="AA14" t="inlineStr">
         <is>
           <t>The Face</t>
         </is>
@@ -2144,22 +2157,32 @@
       <c r="A15" t="n">
         <v>1981</v>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>platinum</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>ck in2u</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
         <is>
           <t>Willy Vanderperre</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>Mert &amp; Marcus</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>Daria Werbowy</t>
         </is>
       </c>
-      <c r="AE15" t="inlineStr">
+      <c r="AA15" t="inlineStr">
         <is>
           <t>AnOther Man</t>
         </is>
@@ -2169,22 +2192,32 @@
       <c r="A16" t="n">
         <v>1982</v>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>secret obsession</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
         <is>
           <t>Fabien Baron</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>Sam Taylor-Johnson</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>Edie Campbell</t>
         </is>
       </c>
-      <c r="AE16" t="inlineStr">
+      <c r="AA16" t="inlineStr">
         <is>
           <t>GQ</t>
         </is>
@@ -2194,17 +2227,22 @@
       <c r="A17" t="n">
         <v>1983</v>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>beauty</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
         <is>
           <t>Peter Lindbergh</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>Anna Ewers</t>
         </is>
       </c>
-      <c r="AE17" t="inlineStr">
+      <c r="AA17" t="inlineStr">
         <is>
           <t>Vanity Fair</t>
         </is>
@@ -2214,12 +2252,17 @@
       <c r="A18" t="n">
         <v>1984</v>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>forbidden euphoria</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
         <is>
           <t>Helmut Newton</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>Saskia de Brauw</t>
         </is>
@@ -2229,12 +2272,17 @@
       <c r="A19" t="n">
         <v>1985</v>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>encounter</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
         <is>
           <t>Annie Leibovitz</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>Justin Bieber</t>
         </is>
@@ -2244,12 +2292,17 @@
       <c r="A20" t="n">
         <v>1986</v>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>downtown</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
         <is>
           <t>Nick Knight</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>Kendall Jenner</t>
         </is>
@@ -2259,12 +2312,17 @@
       <c r="A21" t="n">
         <v>1987</v>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>reveal</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
         <is>
           <t>Juergen Teller</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t>Bella Hadid</t>
         </is>
@@ -2274,12 +2332,17 @@
       <c r="A22" t="n">
         <v>1988</v>
       </c>
-      <c r="S22" t="inlineStr">
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>endless euphoria</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
         <is>
           <t>Tyrone Lebon</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>Lily-Rose Depp</t>
         </is>
@@ -2289,12 +2352,17 @@
       <c r="A23" t="n">
         <v>1989</v>
       </c>
-      <c r="S23" t="inlineStr">
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>eternity now</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
         <is>
           <t>Lachlan Bailey</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>FKA twigs</t>
         </is>
@@ -2304,12 +2372,17 @@
       <c r="A24" t="n">
         <v>1990</v>
       </c>
-      <c r="S24" t="inlineStr">
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>deep euphoria</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
         <is>
           <t>Cass Bird</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="Q24" t="inlineStr">
         <is>
           <t>Solange</t>
         </is>
@@ -2319,12 +2392,17 @@
       <c r="A25" t="n">
         <v>1991</v>
       </c>
-      <c r="S25" t="inlineStr">
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>ck2</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
         <is>
           <t>Harley Weir</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="Q25" t="inlineStr">
         <is>
           <t>A$AP Rocky</t>
         </is>
@@ -2334,12 +2412,17 @@
       <c r="A26" t="n">
         <v>1992</v>
       </c>
-      <c r="S26" t="inlineStr">
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>ck one gold</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
         <is>
           <t>Daniel Jackson</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="Q26" t="inlineStr">
         <is>
           <t>Kaia Gerber</t>
         </is>
@@ -2349,12 +2432,17 @@
       <c r="A27" t="n">
         <v>1993</v>
       </c>
-      <c r="S27" t="inlineStr">
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>obsessed</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
         <is>
           <t>Niall McInerney</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t>Jeremy Allen White</t>
         </is>
@@ -2364,7 +2452,12 @@
       <c r="A28" t="n">
         <v>1994</v>
       </c>
-      <c r="S28" t="inlineStr">
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>women</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
         <is>
           <t>Sølve Sundsbø</t>
         </is>
@@ -2374,7 +2467,12 @@
       <c r="A29" t="n">
         <v>1995</v>
       </c>
-      <c r="S29" t="inlineStr">
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>eternity air</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
         <is>
           <t>Paolo Roversi</t>
         </is>
@@ -2384,7 +2482,12 @@
       <c r="A30" t="n">
         <v>1996</v>
       </c>
-      <c r="S30" t="inlineStr">
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>defy</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
         <is>
           <t>Collier Schorr</t>
         </is>
@@ -2394,7 +2497,12 @@
       <c r="A31" t="n">
         <v>1997</v>
       </c>
-      <c r="S31" t="inlineStr">
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>ck everyone</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
         <is>
           <t>Ethan James Green</t>
         </is>
@@ -2404,16 +2512,31 @@
       <c r="A32" t="n">
         <v>1998</v>
       </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>ck free</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
         <v>1999</v>
       </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>ck all</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
         <v>2000</v>
       </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>eternity moment</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2547,7 +2670,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="31">
+  <tableParts count="27">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
@@ -2575,10 +2698,6 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId25"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId26"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId27"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId28"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId30"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId31"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rename hosier → hosiery in filename, CSV and Excel
</commit_message>
<xml_diff>
--- a/archive_index.xlsx
+++ b/archive_index.xlsx
@@ -1731,7 +1731,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1985_adv_print_hosier_001</t>
+          <t>1985_adv_print_hosiery_001</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>hosier</t>
+          <t>hosiery</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reclassify 1999_ss collection_004/005 → eyewear_002/003
</commit_message>
<xml_diff>
--- a/archive_index.xlsx
+++ b/archive_index.xlsx
@@ -7046,7 +7046,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>1999_ss_adv_print_collection_004</t>
+          <t>1999_ss_adv_print_collection_menswear_001</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -7072,11 +7072,16 @@
           <t>collection</t>
         </is>
       </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>menswear</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>1999_ss_adv_print_collection_005</t>
+          <t>1999_ss_adv_print_collection_menswear_002</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -7102,11 +7107,16 @@
           <t>collection</t>
         </is>
       </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>menswear</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>1999_ss_adv_print_collection_menswear_001</t>
+          <t>1999_ss_adv_print_eyewear_001</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -7129,19 +7139,14 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>collection</t>
-        </is>
-      </c>
-      <c r="G204" t="inlineStr">
-        <is>
-          <t>menswear</t>
+          <t>eyewear</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>1999_ss_adv_print_collection_menswear_002</t>
+          <t>1999_ss_adv_print_eyewear_002</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -7164,19 +7169,14 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>collection</t>
-        </is>
-      </c>
-      <c r="G205" t="inlineStr">
-        <is>
-          <t>menswear</t>
+          <t>eyewear</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>1999_ss_adv_print_eyewear_001</t>
+          <t>1999_ss_adv_print_eyewear_003</t>
         </is>
       </c>
       <c r="B206" t="n">

</xml_diff>

<commit_message>
Fix 'formen' in search labels; rename obsession_men → obsession_formen
- normalize() helper applies formen→for men everywhere labels are built
- enrichSearchWithArchive and filterResults now use normalize()
- Renamed 1995_ss and 1997_ss obsession_men files/CSV/Excel/dims
</commit_message>
<xml_diff>
--- a/archive_index.xlsx
+++ b/archive_index.xlsx
@@ -3931,7 +3931,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>1995_ss_adv_print_fragrance_obsession_men_001</t>
+          <t>1995_ss_adv_print_fragrance_obsession_formen_001</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -3959,7 +3959,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>obsession_men</t>
+          <t>obsession_formen</t>
         </is>
       </c>
     </row>
@@ -5806,7 +5806,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>1997_ss_adv_print_fragrance_obsession_men_001</t>
+          <t>1997_ss_adv_print_fragrance_obsession_formen_001</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -5834,7 +5834,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>obsession_men</t>
+          <t>obsession_formen</t>
         </is>
       </c>
     </row>

</xml_diff>